<commit_message>
feat: apply soft-fixed translations, sync split JSON/Excel, allow and translate Cooldown to Vietnamese, update master prompts
</commit_message>
<xml_diff>
--- a/mistral_translate_work/split_by_prompt/excel/item/lang_item/lang_item__item__part_0001.xlsx
+++ b/mistral_translate_work/split_by_prompt/excel/item/lang_item/lang_item__item__part_0001.xlsx
@@ -28983,7 +28983,7 @@
       </c>
       <c r="M439" t="inlineStr">
         <is>
-          <t>Cung cấp 1.000 Kinh nghiệm Weapons.</t>
+          <t>Cung cấp 1.000 Kinh nghiệm Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -29178,7 +29178,7 @@
       </c>
       <c r="M442" t="inlineStr">
         <is>
-          <t>Cung cấp 3.000 Kinh nghiệm Weapons.</t>
+          <t>Cung cấp 3.000 Kinh nghiệm Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -29373,7 +29373,7 @@
       </c>
       <c r="M445" t="inlineStr">
         <is>
-          <t>Cung cấp 8.000 Kinh nghiệm Weapons.</t>
+          <t>Cung cấp 8.000 Kinh nghiệm Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -29568,7 +29568,7 @@
       </c>
       <c r="M448" t="inlineStr">
         <is>
-          <t>Cung cấp 20.000 Kinh nghiệm Weapons.</t>
+          <t>Cung cấp 20.000 Kinh nghiệm Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -29763,7 +29763,7 @@
       </c>
       <c r="M451" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -29958,7 +29958,7 @@
       </c>
       <c r="M454" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -30153,7 +30153,7 @@
       </c>
       <c r="M457" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -30348,7 +30348,7 @@
       </c>
       <c r="M460" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -30543,7 +30543,7 @@
       </c>
       <c r="M463" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -30738,7 +30738,7 @@
       </c>
       <c r="M466" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -30933,7 +30933,7 @@
       </c>
       <c r="M469" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -31128,7 +31128,7 @@
       </c>
       <c r="M472" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -31323,7 +31323,7 @@
       </c>
       <c r="M475" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -31518,7 +31518,7 @@
       </c>
       <c r="M478" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -31713,7 +31713,7 @@
       </c>
       <c r="M481" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -31908,7 +31908,7 @@
       </c>
       <c r="M484" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -32103,7 +32103,7 @@
       </c>
       <c r="M487" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -32298,7 +32298,7 @@
       </c>
       <c r="M490" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -32493,7 +32493,7 @@
       </c>
       <c r="M493" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -32688,7 +32688,7 @@
       </c>
       <c r="M496" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>
@@ -32883,7 +32883,7 @@
       </c>
       <c r="M499" t="inlineStr">
         <is>
-          <t>Vật phẩm dùng để thăng cấp Weapons.</t>
+          <t>Vật phẩm dùng để thăng cấp Vũ khí.</t>
         </is>
       </c>
     </row>

</xml_diff>